<commit_message>
updated file from Analisis
</commit_message>
<xml_diff>
--- a/Desarrollo/Sistema de Control de Peso (SISCOP)/Analisis/SISCOP-CP.xlsx
+++ b/Desarrollo/Sistema de Control de Peso (SISCOP)/Analisis/SISCOP-CP.xlsx
@@ -483,7 +483,7 @@
     <t>Corregir conflictos y commits pendientes</t>
   </si>
   <si>
-    <t>Hito 3: Desarrollo y Despliegue</t>
+    <t>Hito 3: Desarrollo</t>
   </si>
   <si>
     <t>Realizar pruebas funcionales</t>
@@ -1053,7 +1053,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
@@ -1061,8 +1061,10 @@
     <col customWidth="1" min="2" max="2" width="45.86"/>
     <col customWidth="1" min="3" max="3" width="52.86"/>
     <col customWidth="1" min="4" max="4" width="22.86"/>
-    <col customWidth="1" min="5" max="5" width="87.29"/>
-    <col customWidth="1" min="6" max="8" width="17.29"/>
+    <col customWidth="1" min="5" max="5" width="63.57"/>
+    <col customWidth="1" min="6" max="6" width="13.86"/>
+    <col customWidth="1" min="7" max="7" width="14.0"/>
+    <col customWidth="1" min="8" max="8" width="14.71"/>
     <col customWidth="1" min="9" max="26" width="10.71"/>
   </cols>
   <sheetData>
@@ -2320,7 +2322,7 @@
         <v>46149.0</v>
       </c>
       <c r="G33" s="18">
-        <v>46158.0</v>
+        <v>46159.0</v>
       </c>
       <c r="H33" s="25">
         <v>1.0</v>
@@ -2595,7 +2597,7 @@
         <v>46161.0</v>
       </c>
       <c r="H40" s="23">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
@@ -2667,7 +2669,7 @@
         <v>46163.0</v>
       </c>
       <c r="H42" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
@@ -2709,7 +2711,7 @@
         <v>46165.0</v>
       </c>
       <c r="H43" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I43" s="3"/>
       <c r="J43" s="3"/>
@@ -2751,7 +2753,7 @@
         <v>46170.0</v>
       </c>
       <c r="H44" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
@@ -2793,7 +2795,7 @@
         <v>46171.0</v>
       </c>
       <c r="H45" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
@@ -2835,7 +2837,7 @@
         <v>46167.0</v>
       </c>
       <c r="H46" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
@@ -2877,7 +2879,7 @@
         <v>46172.0</v>
       </c>
       <c r="H47" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
@@ -2919,7 +2921,7 @@
         <v>46175.0</v>
       </c>
       <c r="H48" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
@@ -2991,7 +2993,7 @@
         <v>46164.0</v>
       </c>
       <c r="H50" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I50" s="3"/>
       <c r="J50" s="3"/>
@@ -3033,7 +3035,7 @@
         <v>46166.0</v>
       </c>
       <c r="H51" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
@@ -3075,7 +3077,7 @@
         <v>46169.0</v>
       </c>
       <c r="H52" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
@@ -3117,7 +3119,7 @@
         <v>46171.0</v>
       </c>
       <c r="H53" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I53" s="3"/>
       <c r="J53" s="3"/>
@@ -3159,7 +3161,7 @@
         <v>46173.0</v>
       </c>
       <c r="H54" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I54" s="3"/>
       <c r="J54" s="3"/>
@@ -3201,7 +3203,7 @@
         <v>46175.0</v>
       </c>
       <c r="H55" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I55" s="3"/>
       <c r="J55" s="3"/>
@@ -3239,7 +3241,7 @@
         <v>46176.0</v>
       </c>
       <c r="H56" s="23">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I56" s="3"/>
       <c r="J56" s="3"/>
@@ -3277,7 +3279,7 @@
         <v>46177.0</v>
       </c>
       <c r="H57" s="23">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I57" s="3"/>
       <c r="J57" s="3"/>
@@ -3300,7 +3302,7 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="1"/>
-      <c r="B58" s="34" t="s">
+      <c r="B58" s="27" t="s">
         <v>155</v>
       </c>
       <c r="C58" s="28">
@@ -3351,7 +3353,7 @@
         <v>46180.0</v>
       </c>
       <c r="H59" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I59" s="3"/>
       <c r="J59" s="3"/>
@@ -3387,13 +3389,13 @@
         <v>163</v>
       </c>
       <c r="F60" s="18">
-        <v>46183.0</v>
+        <v>46181.0</v>
       </c>
       <c r="G60" s="18">
         <v>46185.0</v>
       </c>
       <c r="H60" s="25">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I60" s="3"/>
       <c r="J60" s="3"/>
@@ -3432,10 +3434,10 @@
         <v>46185.0</v>
       </c>
       <c r="G61" s="38">
-        <v>46187.0</v>
+        <v>46188.0</v>
       </c>
       <c r="H61" s="41">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I61" s="3"/>
       <c r="J61" s="3"/>
@@ -30654,7 +30656,7 @@
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup fitToHeight="0" paperSize="9" orientation="landscape"/>
   <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>